<commit_message>
feat: actualizar plantilla de excel lote
</commit_message>
<xml_diff>
--- a/pesaje/analytica/Report/Lote-Export-Pesaje-Base.xlsx
+++ b/pesaje/analytica/Report/Lote-Export-Pesaje-Base.xlsx
@@ -8,14 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\projects\minersoft-projects\minersoft\acopio-project-configuration\pesaje\analytica\Report\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F12EFB4C-D3A6-4654-9680-2817304F91BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{03FD3369-30F1-4E98-B83A-661D09834220}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0" iterateDelta="1E-4"/>
+  <calcPr calcId="0"/>
   <extLst>
     <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
       <loext:extCalcPr stringRefSyntax="ExcelA1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="30">
   <si>
     <t>Analytica Mineral Services Sac</t>
   </si>
@@ -102,9 +102,6 @@
     <t>CONDUCTOR</t>
   </si>
   <si>
-    <t>UNIDAD</t>
-  </si>
-  <si>
     <t>PESO BRUTO</t>
   </si>
   <si>
@@ -112,6 +109,12 @@
   </si>
   <si>
     <t>PESO NETO</t>
+  </si>
+  <si>
+    <t>ENVASE</t>
+  </si>
+  <si>
+    <t>SACOS SEGÚN MINERO</t>
   </si>
 </sst>
 </file>
@@ -284,14 +287,14 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="22" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="22" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="24">
@@ -577,7 +580,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AX11"/>
+  <dimension ref="A1:AY11"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="13.6640625" style="4" customWidth="1"/>
@@ -587,13 +590,13 @@
     <col min="5" max="5" width="23.88671875" style="4" customWidth="1"/>
     <col min="6" max="6" width="28.44140625" style="4" customWidth="1"/>
     <col min="7" max="7" width="25.77734375" style="4" customWidth="1"/>
-    <col min="8" max="8" width="28.5546875" style="4" customWidth="1"/>
-    <col min="9" max="9" width="24.77734375" style="4" customWidth="1"/>
-    <col min="10" max="10" width="14.88671875" style="4" customWidth="1"/>
-    <col min="11" max="25" width="24.6640625" style="4" customWidth="1"/>
+    <col min="8" max="9" width="28.5546875" style="4" customWidth="1"/>
+    <col min="10" max="10" width="24.77734375" style="4" customWidth="1"/>
+    <col min="11" max="11" width="14.88671875" style="4" customWidth="1"/>
+    <col min="12" max="26" width="24.6640625" style="4" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:50" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:51" x14ac:dyDescent="0.3">
       <c r="A1" s="5"/>
       <c r="B1" s="5"/>
       <c r="C1" s="5"/>
@@ -619,7 +622,7 @@
       <c r="W1" s="5"/>
       <c r="X1" s="5"/>
       <c r="Y1" s="5"/>
-      <c r="Z1" s="1"/>
+      <c r="Z1" s="5"/>
       <c r="AA1" s="1"/>
       <c r="AB1" s="1"/>
       <c r="AC1" s="1"/>
@@ -644,22 +647,23 @@
       <c r="AV1" s="1"/>
       <c r="AW1" s="1"/>
       <c r="AX1" s="1"/>
+      <c r="AY1" s="1"/>
     </row>
-    <row r="2" spans="1:50" ht="48.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="12" t="s">
+    <row r="2" spans="1:51" ht="48.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="13" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="12"/>
-      <c r="C2" s="12"/>
-      <c r="D2" s="12"/>
-      <c r="E2" s="12"/>
-      <c r="F2" s="12"/>
-      <c r="G2" s="12"/>
-      <c r="H2" s="12"/>
-      <c r="I2" s="12"/>
-      <c r="J2" s="6"/>
+      <c r="B2" s="13"/>
+      <c r="C2" s="13"/>
+      <c r="D2" s="13"/>
+      <c r="E2" s="13"/>
+      <c r="F2" s="13"/>
+      <c r="G2" s="13"/>
+      <c r="H2" s="13"/>
+      <c r="I2" s="13"/>
+      <c r="J2" s="13"/>
       <c r="K2" s="6"/>
-      <c r="L2" s="5"/>
+      <c r="L2" s="6"/>
       <c r="M2" s="5"/>
       <c r="N2" s="5"/>
       <c r="O2" s="5"/>
@@ -673,7 +677,7 @@
       <c r="W2" s="5"/>
       <c r="X2" s="5"/>
       <c r="Y2" s="5"/>
-      <c r="Z2" s="1"/>
+      <c r="Z2" s="5"/>
       <c r="AA2" s="1"/>
       <c r="AB2" s="1"/>
       <c r="AC2" s="1"/>
@@ -698,22 +702,23 @@
       <c r="AV2" s="1"/>
       <c r="AW2" s="1"/>
       <c r="AX2" s="1"/>
+      <c r="AY2" s="1"/>
     </row>
-    <row r="3" spans="1:50" ht="22.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="13" t="s">
+    <row r="3" spans="1:51" ht="22.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="14" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="13"/>
-      <c r="C3" s="13"/>
-      <c r="D3" s="13"/>
-      <c r="E3" s="13"/>
-      <c r="F3" s="13"/>
-      <c r="G3" s="13"/>
-      <c r="H3" s="13"/>
-      <c r="I3" s="13"/>
-      <c r="J3" s="7"/>
+      <c r="B3" s="14"/>
+      <c r="C3" s="14"/>
+      <c r="D3" s="14"/>
+      <c r="E3" s="14"/>
+      <c r="F3" s="14"/>
+      <c r="G3" s="14"/>
+      <c r="H3" s="14"/>
+      <c r="I3" s="14"/>
+      <c r="J3" s="14"/>
       <c r="K3" s="7"/>
-      <c r="L3" s="5"/>
+      <c r="L3" s="7"/>
       <c r="M3" s="5"/>
       <c r="N3" s="5"/>
       <c r="O3" s="5"/>
@@ -727,7 +732,7 @@
       <c r="W3" s="5"/>
       <c r="X3" s="5"/>
       <c r="Y3" s="5"/>
-      <c r="Z3" s="1"/>
+      <c r="Z3" s="5"/>
       <c r="AA3" s="1"/>
       <c r="AB3" s="1"/>
       <c r="AC3" s="1"/>
@@ -752,8 +757,9 @@
       <c r="AV3" s="1"/>
       <c r="AW3" s="1"/>
       <c r="AX3" s="1"/>
+      <c r="AY3" s="1"/>
     </row>
-    <row r="4" spans="1:50" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:51" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="6"/>
       <c r="B4" s="6"/>
       <c r="C4" s="6"/>
@@ -764,7 +770,7 @@
       <c r="H4" s="6"/>
       <c r="I4" s="6"/>
       <c r="J4" s="6"/>
-      <c r="K4" s="5"/>
+      <c r="K4" s="6"/>
       <c r="L4" s="5"/>
       <c r="M4" s="5"/>
       <c r="N4" s="5"/>
@@ -779,7 +785,7 @@
       <c r="W4" s="5"/>
       <c r="X4" s="5"/>
       <c r="Y4" s="5"/>
-      <c r="Z4" s="1"/>
+      <c r="Z4" s="5"/>
       <c r="AA4" s="1"/>
       <c r="AB4" s="1"/>
       <c r="AC4" s="1"/>
@@ -804,8 +810,9 @@
       <c r="AV4" s="1"/>
       <c r="AW4" s="1"/>
       <c r="AX4" s="1"/>
+      <c r="AY4" s="1"/>
     </row>
-    <row r="5" spans="1:50" ht="18" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:51" ht="18" x14ac:dyDescent="0.3">
       <c r="A5" s="8"/>
       <c r="B5" s="8"/>
       <c r="C5" s="8"/>
@@ -816,23 +823,24 @@
       <c r="H5" s="8"/>
       <c r="I5" s="8"/>
       <c r="J5" s="8"/>
-      <c r="K5" s="9"/>
+      <c r="K5" s="8"/>
+      <c r="L5" s="9"/>
     </row>
-    <row r="6" spans="1:50" ht="18" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:51" ht="18" x14ac:dyDescent="0.3">
       <c r="A6" s="9"/>
       <c r="B6" s="10" t="s">
         <v>2</v>
       </c>
-      <c r="C6" s="14"/>
+      <c r="C6" s="12"/>
       <c r="D6" s="9"/>
       <c r="E6" s="9"/>
       <c r="F6" s="9"/>
       <c r="G6" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="K6" s="9"/>
+      <c r="L6" s="9"/>
     </row>
-    <row r="7" spans="1:50" ht="18" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:51" ht="18" x14ac:dyDescent="0.3">
       <c r="A7" s="9"/>
       <c r="B7" s="9"/>
       <c r="C7" s="9"/>
@@ -844,8 +852,9 @@
       <c r="I7" s="9"/>
       <c r="J7" s="9"/>
       <c r="K7" s="9"/>
+      <c r="L7" s="9"/>
     </row>
-    <row r="8" spans="1:50" s="11" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:51" s="11" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
         <v>4</v>
       </c>
@@ -870,68 +879,71 @@
       <c r="H8" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="I8" s="3" t="s">
+      <c r="I8" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="J8" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="J8" s="2" t="s">
+      <c r="K8" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="K8" s="2" t="s">
+      <c r="L8" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="L8" s="2" t="s">
+      <c r="M8" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="M8" s="2" t="s">
+      <c r="N8" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="N8" s="2" t="s">
+      <c r="O8" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="O8" s="2" t="s">
+      <c r="P8" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="P8" s="2" t="s">
+      <c r="Q8" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="Q8" s="3" t="s">
+      <c r="R8" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="R8" s="2" t="s">
+      <c r="S8" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="S8" s="2" t="s">
+      <c r="T8" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="T8" s="2" t="s">
+      <c r="U8" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="U8" s="2" t="s">
+      <c r="V8" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="W8" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="V8" s="2" t="s">
+      <c r="X8" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="W8" s="2" t="s">
+      <c r="Y8" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="X8" s="2" t="s">
+      <c r="Z8" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="Y8" s="2" t="s">
-        <v>7</v>
-      </c>
     </row>
-    <row r="9" spans="1:50" s="4" customFormat="1" x14ac:dyDescent="0.3"/>
-    <row r="11" spans="1:50" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:51" s="4" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="11" spans="1:51" x14ac:dyDescent="0.3">
       <c r="F11" s="4" t="s">
         <v>9</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A2:I2"/>
-    <mergeCell ref="A3:I3"/>
+    <mergeCell ref="A2:J2"/>
+    <mergeCell ref="A3:J3"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>

</xml_diff>

<commit_message>
feat: actualizar plantilla de lote excel
</commit_message>
<xml_diff>
--- a/pesaje/analytica/Report/Lote-Export-Pesaje-Base.xlsx
+++ b/pesaje/analytica/Report/Lote-Export-Pesaje-Base.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\projects\minersoft-projects\minersoft\acopio-project-configuration\pesaje\analytica\Report\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C2E6CCD1-6A7D-4614-8FBA-9AB092830526}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E3841D79-160B-4480-9F1B-326A80C28B26}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="30">
   <si>
     <t>Analytica Mineral Services Sac</t>
   </si>
@@ -109,6 +109,12 @@
   </si>
   <si>
     <t>SACOS SEGÚN MINERO</t>
+  </si>
+  <si>
+    <t>ESTADO ACTA DE CONFORMIDAD</t>
+  </si>
+  <si>
+    <t>NUMERO ACTA CONFORMIDAD</t>
   </si>
 </sst>
 </file>
@@ -588,6 +594,8 @@
     <col min="10" max="10" width="24.77734375" style="4" customWidth="1"/>
     <col min="11" max="11" width="14.88671875" style="4" customWidth="1"/>
     <col min="12" max="24" width="24.6640625" style="4" customWidth="1"/>
+    <col min="25" max="25" width="42.77734375" customWidth="1"/>
+    <col min="26" max="26" width="40.33203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:49" x14ac:dyDescent="0.3">
@@ -910,6 +918,12 @@
       <c r="X8" s="2" t="s">
         <v>26</v>
       </c>
+      <c r="Y8" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="Z8" s="2" t="s">
+        <v>29</v>
+      </c>
     </row>
     <row r="9" spans="1:49" s="4" customFormat="1" x14ac:dyDescent="0.3"/>
     <row r="11" spans="1:49" x14ac:dyDescent="0.3">

</xml_diff>